<commit_message>
feat(cycle-lm): stabilize CYCLE-LM execution state machine, hedge circuit breaker, and UI latency display
- CYCLE-LIMIT-MARKET (CYCLE-LM): Implemented hybrid limit-close / market-reopen strategy mode with strict broker TP confirmation gating and stale flag purge on mode transitions.
- Hedge Monitor Hardening: Enabled Panic Circuit Breaker for MONITOR mode to pause sessions on >15% position drop desyncs; increased bridge partial-read debounce threshold to 10 polls (~5s).
- Execution Latency Fixes: Preserved batch dispatch timestamps across all fills in CYCLE-LM reopen batches, implemented startup batch cmd_ts backfill migration, and capped UI latency rendering between 0ms and 30,000ms.
- Bridge & Direct Connector: Hardened C# MtBridgeService concurrency locks, throttled stale quote log spam, and stabilized FIX/MT Direct account managers.
- Dashboard & UI: Standardized natural account sorting, template-governed rollover day counting, and strategy row persistence.
</commit_message>
<xml_diff>
--- a/Hedge_Optimization_Calculator.xlsx
+++ b/Hedge_Optimization_Calculator.xlsx
@@ -8,12 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="d:\Documents\dev\TradeDashboard\TradeDashboardPY\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5FF64274-1BBE-4DD2-8DBF-CBBA9F10182F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A1979BB8-B8B9-4155-BD12-1E2D37636FF2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="14016" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1140" yWindow="1140" windowWidth="16040" windowHeight="8220" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Hedge Optimization" sheetId="1" r:id="rId1"/>
+    <sheet name="Swaps" sheetId="3" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -33,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="16">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="29">
   <si>
     <t>Hedge Capital Optimization Calculator</t>
   </si>
@@ -62,12 +63,6 @@
     <t>Optimized Allocation</t>
   </si>
   <si>
-    <t>Optimal Alloc. Acc 1 (IC)</t>
-  </si>
-  <si>
-    <t>Optimal Alloc. Acc 2 (YCM)</t>
-  </si>
-  <si>
     <t>Allocation Ratio</t>
   </si>
   <si>
@@ -81,6 +76,51 @@
   </si>
   <si>
     <t>Ratio Acc 2 (+SWAP)</t>
+  </si>
+  <si>
+    <t>YCM</t>
+  </si>
+  <si>
+    <t>usdchf</t>
+  </si>
+  <si>
+    <t>100:1</t>
+  </si>
+  <si>
+    <t>400:1</t>
+  </si>
+  <si>
+    <t>200:1</t>
+  </si>
+  <si>
+    <t>SWP IN POINTS</t>
+  </si>
+  <si>
+    <t>SWP IN USD</t>
+  </si>
+  <si>
+    <t>MAX LEVERAGE</t>
+  </si>
+  <si>
+    <t>MEXATLANTIC</t>
+  </si>
+  <si>
+    <t>DUKASCOPY</t>
+  </si>
+  <si>
+    <t>SWISSQUOTE</t>
+  </si>
+  <si>
+    <t>BRITANNIA</t>
+  </si>
+  <si>
+    <t>as of june 24,2026</t>
+  </si>
+  <si>
+    <t>Optimal Alloc. Acc 1 (SFREE)</t>
+  </si>
+  <si>
+    <t>Optimal Alloc. Acc 2 (+SWAP)</t>
   </si>
 </sst>
 </file>
@@ -90,7 +130,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="\$#,##0.00"/>
   </numFmts>
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -103,6 +143,14 @@
       <sz val="11"/>
       <color rgb="FFFFFFFF"/>
       <name val="Calibri"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="3">
@@ -131,12 +179,15 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="2" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -440,35 +491,35 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:B23"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="32" customWidth="1"/>
     <col min="2" max="2" width="25" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="1"/>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>1</v>
       </c>
       <c r="B2" s="2">
-        <v>2468000</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
+        <v>50000</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>2</v>
       </c>
       <c r="B3">
-        <v>1000</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>3</v>
       </c>
@@ -476,30 +527,30 @@
         <v>100000</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>4</v>
       </c>
       <c r="B5" s="2">
         <f>B3*B4</f>
-        <v>100000000</v>
-      </c>
-    </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.3">
+        <v>2500000</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A7" s="1" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="B7" s="1"/>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>5</v>
       </c>
       <c r="B8">
-        <v>1000</v>
-      </c>
-    </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.3">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>6</v>
       </c>
@@ -507,30 +558,30 @@
         <v>0.5</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>7</v>
       </c>
       <c r="B10" s="2">
         <f>B5*(B9/B8)</f>
-        <v>50000</v>
-      </c>
-    </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.3">
+        <v>12500</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A12" s="1" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="B12" s="1"/>
     </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>5</v>
       </c>
       <c r="B13">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.3">
+        <v>400</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>6</v>
       </c>
@@ -538,64 +589,171 @@
         <v>0.8</v>
       </c>
     </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>7</v>
       </c>
       <c r="B15" s="2">
         <f>B5*(B14/B13)</f>
-        <v>800000</v>
-      </c>
-    </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.3">
+        <v>5000</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A17" s="1" t="s">
         <v>8</v>
       </c>
       <c r="B17" s="1"/>
     </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
-        <v>9</v>
+        <v>27</v>
       </c>
       <c r="B18" s="2">
         <f>(B2/2)+((B10-B15)/2)</f>
-        <v>859000</v>
-      </c>
-    </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.3">
+        <v>28750</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
-        <v>10</v>
+        <v>28</v>
       </c>
       <c r="B19" s="2">
         <f>(B2/2)-((B10-B15)/2)</f>
-        <v>1609000</v>
-      </c>
-    </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.3">
+        <v>21250</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A21" s="1" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="B21" s="1"/>
     </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B22" s="4">
         <f>B18/B2</f>
-        <v>0.34805510534846029</v>
-      </c>
-    </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.3">
+        <v>0.57499999999999996</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="B23" s="4">
         <f>B19/B2</f>
-        <v>0.65194489465153971</v>
+        <v>0.42499999999999999</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D5E03EE0-2349-4BB4-89F2-581C4FD197A5}">
+  <dimension ref="A1:H5"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="13.453125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="9.90625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="10.90625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="11.90625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="11.81640625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="B1" t="s">
+        <v>25</v>
+      </c>
+      <c r="C1" t="s">
+        <v>23</v>
+      </c>
+      <c r="D1" t="s">
+        <v>24</v>
+      </c>
+      <c r="E1" t="s">
+        <v>14</v>
+      </c>
+      <c r="F1" t="s">
+        <v>22</v>
+      </c>
+      <c r="H1" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>21</v>
+      </c>
+      <c r="B2" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="C2" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="D2" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="E2" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="F2" s="5" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>19</v>
+      </c>
+      <c r="B3">
+        <v>7.86</v>
+      </c>
+      <c r="C3">
+        <v>7.6</v>
+      </c>
+      <c r="E3">
+        <v>7.1</v>
+      </c>
+      <c r="F3">
+        <v>6.36</v>
+      </c>
+      <c r="H3">
+        <v>0.81799999999999995</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
+        <v>20</v>
+      </c>
+      <c r="B4" s="6">
+        <f>B3/$H$3</f>
+        <v>9.6088019559902218</v>
+      </c>
+      <c r="C4" s="6">
+        <f>C3/$H$3</f>
+        <v>9.2909535452322736</v>
+      </c>
+      <c r="D4" s="7">
+        <v>8.85</v>
+      </c>
+      <c r="E4" s="6">
+        <f>E3/$H$3</f>
+        <v>8.679706601466993</v>
+      </c>
+      <c r="F4" s="6">
+        <f>F3/$H$3</f>
+        <v>7.7750611246943775</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="B5" t="s">
+        <v>26</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="360" verticalDpi="360" r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>